<commit_message>
Add legend for pipelines not inluded
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/outputs_IAEE_2025_run_2024_utilization_share.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/outputs_IAEE_2025_run_2024_utilization_share.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,11 +449,6 @@
           <t>Share</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -470,11 +465,6 @@
       <c r="D2" t="n">
         <v>0.9323264308816184</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -491,11 +481,6 @@
       <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -512,11 +497,6 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -533,11 +513,6 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -554,11 +529,6 @@
       <c r="D6" t="n">
         <v>0.2486293875059008</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -575,11 +545,6 @@
       <c r="D7" t="n">
         <v>0.2654259259259258</v>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -596,11 +561,6 @@
       <c r="D8" t="n">
         <v>0.9264787133407526</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -617,11 +577,6 @@
       <c r="D9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -638,11 +593,6 @@
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -659,11 +609,6 @@
       <c r="D11" t="n">
         <v>0.8263845589787139</v>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -680,11 +625,6 @@
       <c r="D12" t="n">
         <v>0.9337363794779939</v>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -701,11 +641,6 @@
       <c r="D13" t="n">
         <v>0.7579979174921611</v>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -722,11 +657,6 @@
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -743,11 +673,6 @@
       <c r="D15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -764,11 +689,6 @@
       <c r="D16" t="n">
         <v>0.5895383241025784</v>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -785,11 +705,6 @@
       <c r="D17" t="n">
         <v>0.3160412107339819</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -806,11 +721,6 @@
       <c r="D18" t="n">
         <v>0.1928450755506194</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>royalblue</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -827,11 +737,6 @@
       <c r="D19" t="n">
         <v>0.5051922897104595</v>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -847,11 +752,6 @@
       </c>
       <c r="D20" t="n">
         <v>0.6118668095510167</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>